<commit_message>
Feat: FERC reference CSV integration (v0.1c)
- Add tools/extract_ferc_pdf.py for one-time PDF extraction
- Add requirements-dev.txt (pdfplumber, dev-only)
- Auto-detect resources/ferc_uniform_system.csv on startup in cli.py
- Add _parse_business_unit_sheet() to loader.py for non-standard BU sheet layout
- Add bu_type parameter to placer.py score_parent_candidates() for exact BU filtering
- Fix suggester.py fill_defaults() reasoning overwrite bug
- Update CHANGELOG.md to v0.1c
</commit_message>
<xml_diff>
--- a/resources/Silver_Dolphins_CoA.xlsx
+++ b/resources/Silver_Dolphins_CoA.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mkc53\ClaudeProjects\Silver_Dolphins_AUDIT\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mkc53\ClaudeProjects\Silver_Dolphins_AUDIT\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A2888EB-A0D8-4EE1-BB1E-0148179BC4C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FF0AB64-CEFB-4718-A08C-7165C51E47E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21840" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Chart of Accounts" sheetId="1" r:id="rId1"/>
@@ -25,15 +25,28 @@
     <sheet name="Cash Flow Category" sheetId="10" r:id="rId10"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Chart of Accounts'!$A$1:$L$99</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Chart of Accounts'!$A$1:$L$120</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'FERC Code'!$A$9:$C$71</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="498" uniqueCount="345">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="541" uniqueCount="369">
   <si>
     <t>Account ID</t>
   </si>
@@ -1068,6 +1081,78 @@
   </si>
   <si>
     <t>Net Position - End of Year</t>
+  </si>
+  <si>
+    <t>Executives</t>
+  </si>
+  <si>
+    <t>Energy Transmission</t>
+  </si>
+  <si>
+    <t>Electric Production</t>
+  </si>
+  <si>
+    <t>Electric Transmission</t>
+  </si>
+  <si>
+    <t>Retail Electric Revenues</t>
+  </si>
+  <si>
+    <t>Resale Electric Revenues</t>
+  </si>
+  <si>
+    <t>Other Revenues</t>
+  </si>
+  <si>
+    <t>Fuel and Purchased Power</t>
+  </si>
+  <si>
+    <t>Operation and Maintenance</t>
+  </si>
+  <si>
+    <t>Depr and Amort Expense</t>
+  </si>
+  <si>
+    <t>Propert and Other Taxes</t>
+  </si>
+  <si>
+    <t>General and Administrative</t>
+  </si>
+  <si>
+    <t>Regulatory Amortization</t>
+  </si>
+  <si>
+    <t>Other Operating Expenses</t>
+  </si>
+  <si>
+    <t>Other Non Operating Income</t>
+  </si>
+  <si>
+    <t>Interest Income</t>
+  </si>
+  <si>
+    <t>Investment Income</t>
+  </si>
+  <si>
+    <t>Rental and Lease Income</t>
+  </si>
+  <si>
+    <t>Interest Expense</t>
+  </si>
+  <si>
+    <t>Loss on Sale of Assets</t>
+  </si>
+  <si>
+    <t>Debt Issuance Costs</t>
+  </si>
+  <si>
+    <t>Impairment Charges</t>
+  </si>
+  <si>
+    <t>Other Special Items</t>
+  </si>
+  <si>
+    <t>Special Items</t>
   </si>
 </sst>
 </file>
@@ -1333,10 +1418,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1349,6 +1430,10 @@
       <alignment indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1694,7 +1779,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L100"/>
+  <dimension ref="A1:L120"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.7109375" bestFit="1" customWidth="1"/>
@@ -1951,7 +2036,7 @@
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B9">
         <v>10</v>
@@ -1983,13 +2068,13 @@
     </row>
     <row r="10" spans="1:12" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B10">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C10">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="D10" t="s">
         <v>12</v>
@@ -2009,13 +2094,13 @@
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B11">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="C11">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="D11" t="s">
         <v>12</v>
@@ -2035,7 +2120,7 @@
     </row>
     <row r="12" spans="1:12" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B12">
         <v>10</v>
@@ -2061,7 +2146,7 @@
     </row>
     <row r="13" spans="1:12" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B13">
         <v>10</v>
@@ -2090,7 +2175,7 @@
     </row>
     <row r="14" spans="1:12" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B14">
         <v>10</v>
@@ -2119,7 +2204,7 @@
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B15">
         <v>10</v>
@@ -2145,7 +2230,7 @@
     </row>
     <row r="16" spans="1:12" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B16">
         <v>10</v>
@@ -2171,7 +2256,7 @@
     </row>
     <row r="17" spans="1:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B17">
         <v>10</v>
@@ -2197,7 +2282,7 @@
     </row>
     <row r="18" spans="1:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B18">
         <v>10</v>
@@ -2223,7 +2308,7 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B19">
         <v>10</v>
@@ -2252,7 +2337,7 @@
     </row>
     <row r="20" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B20">
         <v>10</v>
@@ -2278,7 +2363,7 @@
     </row>
     <row r="21" spans="1:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B21">
         <v>10</v>
@@ -2307,7 +2392,7 @@
     </row>
     <row r="22" spans="1:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B22">
         <v>10</v>
@@ -2333,7 +2418,7 @@
     </row>
     <row r="23" spans="1:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B23">
         <v>10</v>
@@ -2359,7 +2444,7 @@
     </row>
     <row r="24" spans="1:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B24">
         <v>10</v>
@@ -2385,7 +2470,7 @@
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B25">
         <v>10</v>
@@ -2411,7 +2496,7 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B26">
         <v>10</v>
@@ -2440,7 +2525,7 @@
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B27">
         <v>10</v>
@@ -2469,7 +2554,7 @@
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B28">
         <v>10</v>
@@ -2495,7 +2580,7 @@
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B29">
         <v>10</v>
@@ -2521,7 +2606,7 @@
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B30">
         <v>10</v>
@@ -2550,7 +2635,7 @@
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B31">
         <v>10</v>
@@ -2576,7 +2661,7 @@
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B32">
         <v>10</v>
@@ -2602,7 +2687,7 @@
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B33">
         <v>10</v>
@@ -2631,7 +2716,7 @@
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B34">
         <v>10</v>
@@ -2657,7 +2742,7 @@
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B35">
         <v>10</v>
@@ -2683,7 +2768,7 @@
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B36">
         <v>10</v>
@@ -2709,7 +2794,7 @@
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B37">
         <v>10</v>
@@ -2735,7 +2820,7 @@
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B38">
         <v>10</v>
@@ -2761,7 +2846,7 @@
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B39">
         <v>10</v>
@@ -2790,7 +2875,7 @@
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B40">
         <v>10</v>
@@ -2819,7 +2904,7 @@
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B41">
         <v>10</v>
@@ -2848,7 +2933,7 @@
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B42">
         <v>10</v>
@@ -2874,7 +2959,7 @@
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B43">
         <v>10</v>
@@ -2900,7 +2985,7 @@
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B44">
         <v>10</v>
@@ -2926,7 +3011,7 @@
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B45">
         <v>10</v>
@@ -2952,7 +3037,7 @@
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B46">
         <v>10</v>
@@ -2978,7 +3063,7 @@
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B47">
         <v>10</v>
@@ -3004,7 +3089,7 @@
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B48">
         <v>10</v>
@@ -3030,7 +3115,7 @@
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B49">
         <v>10</v>
@@ -3059,7 +3144,7 @@
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B50">
         <v>10</v>
@@ -3085,7 +3170,7 @@
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B51">
         <v>10</v>
@@ -3111,7 +3196,7 @@
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B52">
         <v>10</v>
@@ -3137,7 +3222,7 @@
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B53">
         <v>10</v>
@@ -3163,7 +3248,7 @@
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B54">
         <v>10</v>
@@ -3189,7 +3274,7 @@
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B55">
         <v>10</v>
@@ -3218,7 +3303,7 @@
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B56">
         <v>10</v>
@@ -3247,7 +3332,7 @@
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A57">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B57">
         <v>10</v>
@@ -3273,7 +3358,7 @@
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B58">
         <v>10</v>
@@ -3299,7 +3384,7 @@
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B59">
         <v>10</v>
@@ -3325,7 +3410,7 @@
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B60">
         <v>10</v>
@@ -3351,7 +3436,7 @@
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A61">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B61">
         <v>10</v>
@@ -3380,7 +3465,7 @@
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B62">
         <v>10</v>
@@ -3392,13 +3477,13 @@
         <v>74</v>
       </c>
       <c r="E62">
-        <v>400100</v>
+        <v>400001</v>
       </c>
       <c r="F62" t="s">
-        <v>76</v>
+        <v>349</v>
       </c>
       <c r="H62">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I62">
         <v>440</v>
@@ -3406,33 +3491,33 @@
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A63">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B63">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C63">
-        <v>10000</v>
+        <v>20100</v>
       </c>
       <c r="D63" t="s">
         <v>74</v>
       </c>
       <c r="E63">
-        <v>400200</v>
+        <v>400100</v>
       </c>
       <c r="F63" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H63">
         <v>5</v>
       </c>
       <c r="I63">
-        <v>442</v>
+        <v>440</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A64">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B64">
         <v>10</v>
@@ -3444,10 +3529,10 @@
         <v>74</v>
       </c>
       <c r="E64">
-        <v>400300</v>
+        <v>400200</v>
       </c>
       <c r="F64" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H64">
         <v>5</v>
@@ -3458,7 +3543,7 @@
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A65">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B65">
         <v>10</v>
@@ -3470,10 +3555,10 @@
         <v>74</v>
       </c>
       <c r="E65">
-        <v>401000</v>
+        <v>400300</v>
       </c>
       <c r="F65" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H65">
         <v>5</v>
@@ -3484,7 +3569,7 @@
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A66">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B66">
         <v>10</v>
@@ -3496,21 +3581,21 @@
         <v>74</v>
       </c>
       <c r="E66">
-        <v>420100</v>
+        <v>401000</v>
       </c>
       <c r="F66" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H66">
         <v>5</v>
       </c>
       <c r="I66">
-        <v>447</v>
+        <v>442</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A67">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B67">
         <v>10</v>
@@ -3522,13 +3607,13 @@
         <v>74</v>
       </c>
       <c r="E67">
-        <v>421000</v>
+        <v>420000</v>
       </c>
       <c r="F67" t="s">
-        <v>81</v>
+        <v>350</v>
       </c>
       <c r="H67">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I67">
         <v>447</v>
@@ -3536,7 +3621,7 @@
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A68">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B68">
         <v>10</v>
@@ -3548,21 +3633,21 @@
         <v>74</v>
       </c>
       <c r="E68">
-        <v>450100</v>
+        <v>420100</v>
       </c>
       <c r="F68" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="H68">
         <v>5</v>
       </c>
       <c r="I68">
-        <v>456</v>
+        <v>447</v>
       </c>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A69">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B69">
         <v>10</v>
@@ -3574,21 +3659,21 @@
         <v>74</v>
       </c>
       <c r="E69">
-        <v>451000</v>
+        <v>421000</v>
       </c>
       <c r="F69" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="H69">
         <v>5</v>
       </c>
       <c r="I69">
-        <v>450</v>
+        <v>447</v>
       </c>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A70">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B70">
         <v>10</v>
@@ -3600,24 +3685,21 @@
         <v>74</v>
       </c>
       <c r="E70">
-        <v>500000</v>
+        <v>450000</v>
       </c>
       <c r="F70" t="s">
-        <v>84</v>
-      </c>
-      <c r="G70" t="s">
-        <v>14</v>
+        <v>351</v>
       </c>
       <c r="H70">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I70">
-        <v>501</v>
+        <v>456</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A71">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B71">
         <v>10</v>
@@ -3629,21 +3711,21 @@
         <v>74</v>
       </c>
       <c r="E71">
-        <v>500100</v>
+        <v>450100</v>
       </c>
       <c r="F71" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="H71">
         <v>5</v>
       </c>
       <c r="I71">
-        <v>501</v>
+        <v>456</v>
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A72">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B72">
         <v>10</v>
@@ -3655,21 +3737,21 @@
         <v>74</v>
       </c>
       <c r="E72">
-        <v>500200</v>
+        <v>451000</v>
       </c>
       <c r="F72" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="H72">
         <v>5</v>
       </c>
       <c r="I72">
-        <v>555</v>
+        <v>450</v>
       </c>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A73">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B73">
         <v>10</v>
@@ -3681,13 +3763,16 @@
         <v>74</v>
       </c>
       <c r="E73">
-        <v>501000</v>
+        <v>500000</v>
       </c>
       <c r="F73" t="s">
-        <v>87</v>
+        <v>84</v>
+      </c>
+      <c r="G73" t="s">
+        <v>14</v>
       </c>
       <c r="H73">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I73">
         <v>501</v>
@@ -3695,7 +3780,7 @@
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A74">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B74">
         <v>10</v>
@@ -3707,47 +3792,47 @@
         <v>74</v>
       </c>
       <c r="E74">
-        <v>510100</v>
+        <v>500001</v>
       </c>
       <c r="F74" t="s">
-        <v>88</v>
+        <v>352</v>
       </c>
       <c r="H74">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I74">
-        <v>500</v>
+        <v>501</v>
       </c>
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A75">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B75">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C75">
-        <v>10000</v>
+        <v>20100</v>
       </c>
       <c r="D75" t="s">
         <v>74</v>
       </c>
       <c r="E75">
-        <v>511000</v>
+        <v>500100</v>
       </c>
       <c r="F75" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="H75">
         <v>5</v>
       </c>
       <c r="I75">
-        <v>571</v>
+        <v>501</v>
       </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A76">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B76">
         <v>10</v>
@@ -3759,21 +3844,21 @@
         <v>74</v>
       </c>
       <c r="E76">
-        <v>512000</v>
+        <v>500200</v>
       </c>
       <c r="F76" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="H76">
         <v>5</v>
       </c>
       <c r="I76">
-        <v>593</v>
+        <v>555</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A77">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B77">
         <v>10</v>
@@ -3785,21 +3870,21 @@
         <v>74</v>
       </c>
       <c r="E77">
-        <v>515000</v>
+        <v>501000</v>
       </c>
       <c r="F77" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="H77">
         <v>5</v>
       </c>
       <c r="I77">
-        <v>506</v>
+        <v>501</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A78">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B78">
         <v>10</v>
@@ -3811,21 +3896,21 @@
         <v>74</v>
       </c>
       <c r="E78">
-        <v>530100</v>
+        <v>510000</v>
       </c>
       <c r="F78" t="s">
-        <v>92</v>
+        <v>353</v>
       </c>
       <c r="H78">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I78">
-        <v>403</v>
+        <v>501</v>
       </c>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A79">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B79">
         <v>10</v>
@@ -3837,21 +3922,21 @@
         <v>74</v>
       </c>
       <c r="E79">
-        <v>530200</v>
+        <v>510100</v>
       </c>
       <c r="F79" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="H79">
         <v>5</v>
       </c>
       <c r="I79">
-        <v>403</v>
+        <v>500</v>
       </c>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A80">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B80">
         <v>10</v>
@@ -3863,21 +3948,21 @@
         <v>74</v>
       </c>
       <c r="E80">
-        <v>530300</v>
+        <v>511000</v>
       </c>
       <c r="F80" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="H80">
         <v>5</v>
       </c>
       <c r="I80">
-        <v>403</v>
+        <v>571</v>
       </c>
     </row>
     <row r="81" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A81">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B81">
         <v>10</v>
@@ -3889,21 +3974,21 @@
         <v>74</v>
       </c>
       <c r="E81">
-        <v>530400</v>
+        <v>512000</v>
       </c>
       <c r="F81" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="H81">
         <v>5</v>
       </c>
       <c r="I81">
-        <v>403</v>
+        <v>593</v>
       </c>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A82">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B82">
         <v>10</v>
@@ -3915,21 +4000,21 @@
         <v>74</v>
       </c>
       <c r="E82">
-        <v>530500</v>
+        <v>515000</v>
       </c>
       <c r="F82" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="H82">
         <v>5</v>
       </c>
       <c r="I82">
-        <v>404</v>
+        <v>506</v>
       </c>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A83">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B83">
         <v>10</v>
@@ -3941,21 +4026,21 @@
         <v>74</v>
       </c>
       <c r="E83">
-        <v>540100</v>
+        <v>530000</v>
       </c>
       <c r="F83" t="s">
-        <v>97</v>
+        <v>354</v>
       </c>
       <c r="H83">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I83">
-        <v>408.1</v>
+        <v>403</v>
       </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A84">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B84">
         <v>10</v>
@@ -3967,21 +4052,21 @@
         <v>74</v>
       </c>
       <c r="E84">
-        <v>541000</v>
+        <v>530100</v>
       </c>
       <c r="F84" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="H84">
         <v>5</v>
       </c>
       <c r="I84">
-        <v>408.1</v>
+        <v>403</v>
       </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A85">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B85">
         <v>10</v>
@@ -3993,47 +4078,47 @@
         <v>74</v>
       </c>
       <c r="E85">
-        <v>550100</v>
+        <v>530200</v>
       </c>
       <c r="F85" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="H85">
         <v>5</v>
       </c>
       <c r="I85">
-        <v>926</v>
+        <v>403</v>
       </c>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A86">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B86">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="C86">
-        <v>10000</v>
+        <v>30100</v>
       </c>
       <c r="D86" t="s">
         <v>74</v>
       </c>
       <c r="E86">
-        <v>550200</v>
+        <v>530300</v>
       </c>
       <c r="F86" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="H86">
         <v>5</v>
       </c>
       <c r="I86">
-        <v>920</v>
+        <v>403</v>
       </c>
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A87">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B87">
         <v>10</v>
@@ -4045,73 +4130,73 @@
         <v>74</v>
       </c>
       <c r="E87">
-        <v>551000</v>
+        <v>530400</v>
       </c>
       <c r="F87" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="H87">
         <v>5</v>
       </c>
       <c r="I87">
-        <v>923</v>
+        <v>403</v>
       </c>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A88">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B88">
         <v>10</v>
       </c>
       <c r="C88">
-        <v>10000</v>
+        <v>10100</v>
       </c>
       <c r="D88" t="s">
         <v>74</v>
       </c>
       <c r="E88">
-        <v>552000</v>
+        <v>530500</v>
       </c>
       <c r="F88" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="H88">
         <v>5</v>
       </c>
       <c r="I88">
-        <v>920</v>
+        <v>404</v>
       </c>
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A89">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B89">
         <v>10</v>
       </c>
       <c r="C89">
-        <v>10000</v>
+        <v>10100</v>
       </c>
       <c r="D89" t="s">
         <v>74</v>
       </c>
       <c r="E89">
-        <v>553000</v>
+        <v>540000</v>
       </c>
       <c r="F89" t="s">
-        <v>103</v>
+        <v>355</v>
       </c>
       <c r="H89">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I89">
-        <v>921</v>
+        <v>408</v>
       </c>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A90">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B90">
         <v>10</v>
@@ -4123,21 +4208,21 @@
         <v>74</v>
       </c>
       <c r="E90">
-        <v>570100</v>
+        <v>540100</v>
       </c>
       <c r="F90" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="H90">
         <v>5</v>
       </c>
       <c r="I90">
-        <v>407.3</v>
+        <v>408.1</v>
       </c>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A91">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B91">
         <v>10</v>
@@ -4149,24 +4234,21 @@
         <v>74</v>
       </c>
       <c r="E91">
-        <v>600000</v>
+        <v>541000</v>
       </c>
       <c r="F91" t="s">
-        <v>105</v>
-      </c>
-      <c r="G91" t="s">
-        <v>14</v>
+        <v>98</v>
       </c>
       <c r="H91">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I91">
-        <v>419</v>
+        <v>408.1</v>
       </c>
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A92">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B92">
         <v>10</v>
@@ -4178,21 +4260,21 @@
         <v>74</v>
       </c>
       <c r="E92">
-        <v>600100</v>
+        <v>550000</v>
       </c>
       <c r="F92" t="s">
-        <v>106</v>
+        <v>356</v>
       </c>
       <c r="H92">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I92">
-        <v>419</v>
+        <v>920</v>
       </c>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A93">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B93">
         <v>10</v>
@@ -4204,21 +4286,21 @@
         <v>74</v>
       </c>
       <c r="E93">
-        <v>610100</v>
+        <v>550100</v>
       </c>
       <c r="F93" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="H93">
         <v>5</v>
       </c>
       <c r="I93">
-        <v>419</v>
+        <v>926</v>
       </c>
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A94">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B94">
         <v>10</v>
@@ -4230,21 +4312,21 @@
         <v>74</v>
       </c>
       <c r="E94">
-        <v>620100</v>
+        <v>550200</v>
       </c>
       <c r="F94" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="H94">
         <v>5</v>
       </c>
       <c r="I94">
-        <v>418</v>
+        <v>920</v>
       </c>
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A95">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B95">
         <v>10</v>
@@ -4256,24 +4338,21 @@
         <v>74</v>
       </c>
       <c r="E95">
-        <v>700000</v>
+        <v>551000</v>
       </c>
       <c r="F95" t="s">
-        <v>109</v>
-      </c>
-      <c r="G95" t="s">
-        <v>14</v>
+        <v>101</v>
       </c>
       <c r="H95">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I95">
-        <v>421</v>
+        <v>923</v>
       </c>
     </row>
     <row r="96" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A96">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B96">
         <v>10</v>
@@ -4285,21 +4364,21 @@
         <v>74</v>
       </c>
       <c r="E96">
-        <v>700100</v>
+        <v>552000</v>
       </c>
       <c r="F96" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="H96">
         <v>5</v>
       </c>
       <c r="I96">
-        <v>427</v>
+        <v>920</v>
       </c>
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A97">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B97">
         <v>10</v>
@@ -4311,21 +4390,21 @@
         <v>74</v>
       </c>
       <c r="E97">
-        <v>701000</v>
+        <v>553000</v>
       </c>
       <c r="F97" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="H97">
         <v>5</v>
       </c>
       <c r="I97">
-        <v>427</v>
+        <v>921</v>
       </c>
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A98">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B98">
         <v>10</v>
@@ -4337,21 +4416,21 @@
         <v>74</v>
       </c>
       <c r="E98">
-        <v>730100</v>
+        <v>570000</v>
       </c>
       <c r="F98" t="s">
-        <v>112</v>
+        <v>357</v>
       </c>
       <c r="H98">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I98">
-        <v>428</v>
+        <v>501</v>
       </c>
     </row>
     <row r="99" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A99">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B99">
         <v>10</v>
@@ -4363,21 +4442,21 @@
         <v>74</v>
       </c>
       <c r="E99">
-        <v>800100</v>
+        <v>570100</v>
       </c>
       <c r="F99" t="s">
-        <v>113</v>
+        <v>104</v>
       </c>
       <c r="H99">
         <v>5</v>
       </c>
       <c r="I99">
-        <v>426.5</v>
+        <v>407.3</v>
       </c>
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A100">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B100">
         <v>10</v>
@@ -4389,24 +4468,546 @@
         <v>74</v>
       </c>
       <c r="E100">
+        <v>580000</v>
+      </c>
+      <c r="F100" t="s">
+        <v>358</v>
+      </c>
+      <c r="H100">
+        <v>2</v>
+      </c>
+      <c r="I100">
+        <v>999</v>
+      </c>
+    </row>
+    <row r="101" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A101">
+        <v>100</v>
+      </c>
+      <c r="B101">
+        <v>10</v>
+      </c>
+      <c r="C101">
+        <v>10000</v>
+      </c>
+      <c r="D101" t="s">
+        <v>74</v>
+      </c>
+      <c r="E101">
+        <v>600000</v>
+      </c>
+      <c r="F101" t="s">
+        <v>105</v>
+      </c>
+      <c r="G101" t="s">
+        <v>14</v>
+      </c>
+      <c r="H101">
+        <v>1</v>
+      </c>
+      <c r="I101">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="102" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A102">
+        <v>101</v>
+      </c>
+      <c r="B102">
+        <v>10</v>
+      </c>
+      <c r="C102">
+        <v>10000</v>
+      </c>
+      <c r="D102" t="s">
+        <v>74</v>
+      </c>
+      <c r="E102">
+        <v>600001</v>
+      </c>
+      <c r="F102" t="s">
+        <v>360</v>
+      </c>
+      <c r="H102">
+        <v>2</v>
+      </c>
+      <c r="I102">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="103" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A103">
+        <v>102</v>
+      </c>
+      <c r="B103">
+        <v>10</v>
+      </c>
+      <c r="C103">
+        <v>10000</v>
+      </c>
+      <c r="D103" t="s">
+        <v>74</v>
+      </c>
+      <c r="E103">
+        <v>600100</v>
+      </c>
+      <c r="F103" t="s">
+        <v>106</v>
+      </c>
+      <c r="H103">
+        <v>5</v>
+      </c>
+      <c r="I103">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="104" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A104">
+        <v>103</v>
+      </c>
+      <c r="B104">
+        <v>10</v>
+      </c>
+      <c r="C104">
+        <v>10000</v>
+      </c>
+      <c r="D104" t="s">
+        <v>74</v>
+      </c>
+      <c r="E104">
+        <v>610000</v>
+      </c>
+      <c r="F104" t="s">
+        <v>361</v>
+      </c>
+      <c r="H104">
+        <v>2</v>
+      </c>
+      <c r="I104">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="105" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A105">
+        <v>104</v>
+      </c>
+      <c r="B105">
+        <v>10</v>
+      </c>
+      <c r="C105">
+        <v>10000</v>
+      </c>
+      <c r="D105" t="s">
+        <v>74</v>
+      </c>
+      <c r="E105">
+        <v>610100</v>
+      </c>
+      <c r="F105" t="s">
+        <v>107</v>
+      </c>
+      <c r="H105">
+        <v>5</v>
+      </c>
+      <c r="I105">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="106" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A106">
+        <v>105</v>
+      </c>
+      <c r="B106">
+        <v>10</v>
+      </c>
+      <c r="C106">
+        <v>10000</v>
+      </c>
+      <c r="D106" t="s">
+        <v>74</v>
+      </c>
+      <c r="E106">
+        <v>620000</v>
+      </c>
+      <c r="F106" t="s">
+        <v>362</v>
+      </c>
+      <c r="H106">
+        <v>2</v>
+      </c>
+      <c r="I106">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="107" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A107">
+        <v>106</v>
+      </c>
+      <c r="B107">
+        <v>10</v>
+      </c>
+      <c r="C107">
+        <v>10000</v>
+      </c>
+      <c r="D107" t="s">
+        <v>74</v>
+      </c>
+      <c r="E107">
+        <v>620100</v>
+      </c>
+      <c r="F107" t="s">
+        <v>108</v>
+      </c>
+      <c r="H107">
+        <v>5</v>
+      </c>
+      <c r="I107">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="108" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A108">
+        <v>107</v>
+      </c>
+      <c r="B108">
+        <v>10</v>
+      </c>
+      <c r="C108">
+        <v>10000</v>
+      </c>
+      <c r="D108" t="s">
+        <v>74</v>
+      </c>
+      <c r="E108">
+        <v>630000</v>
+      </c>
+      <c r="F108" t="s">
+        <v>359</v>
+      </c>
+      <c r="H108">
+        <v>2</v>
+      </c>
+      <c r="I108">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="109" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A109">
+        <v>108</v>
+      </c>
+      <c r="B109">
+        <v>10</v>
+      </c>
+      <c r="C109">
+        <v>10000</v>
+      </c>
+      <c r="D109" t="s">
+        <v>74</v>
+      </c>
+      <c r="E109">
+        <v>700001</v>
+      </c>
+      <c r="F109" t="s">
+        <v>363</v>
+      </c>
+      <c r="H109">
+        <v>2</v>
+      </c>
+      <c r="I109">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="110" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A110">
+        <v>109</v>
+      </c>
+      <c r="B110">
+        <v>10</v>
+      </c>
+      <c r="C110">
+        <v>10000</v>
+      </c>
+      <c r="D110" t="s">
+        <v>74</v>
+      </c>
+      <c r="E110">
+        <v>700000</v>
+      </c>
+      <c r="F110" t="s">
+        <v>109</v>
+      </c>
+      <c r="G110" t="s">
+        <v>14</v>
+      </c>
+      <c r="H110">
+        <v>1</v>
+      </c>
+      <c r="I110">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="111" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A111">
+        <v>110</v>
+      </c>
+      <c r="B111">
+        <v>10</v>
+      </c>
+      <c r="C111">
+        <v>10000</v>
+      </c>
+      <c r="D111" t="s">
+        <v>74</v>
+      </c>
+      <c r="E111">
+        <v>700100</v>
+      </c>
+      <c r="F111" t="s">
+        <v>110</v>
+      </c>
+      <c r="H111">
+        <v>5</v>
+      </c>
+      <c r="I111">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="112" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A112">
+        <v>111</v>
+      </c>
+      <c r="B112">
+        <v>10</v>
+      </c>
+      <c r="C112">
+        <v>10000</v>
+      </c>
+      <c r="D112" t="s">
+        <v>74</v>
+      </c>
+      <c r="E112">
+        <v>701000</v>
+      </c>
+      <c r="F112" t="s">
+        <v>111</v>
+      </c>
+      <c r="H112">
+        <v>5</v>
+      </c>
+      <c r="I112">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="113" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A113">
+        <v>112</v>
+      </c>
+      <c r="B113">
+        <v>10</v>
+      </c>
+      <c r="C113">
+        <v>10000</v>
+      </c>
+      <c r="D113" t="s">
+        <v>74</v>
+      </c>
+      <c r="E113">
+        <v>720000</v>
+      </c>
+      <c r="F113" t="s">
+        <v>364</v>
+      </c>
+      <c r="H113">
+        <v>2</v>
+      </c>
+      <c r="I113">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="114" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A114">
+        <v>113</v>
+      </c>
+      <c r="B114">
+        <v>10</v>
+      </c>
+      <c r="C114">
+        <v>10000</v>
+      </c>
+      <c r="D114" t="s">
+        <v>74</v>
+      </c>
+      <c r="E114">
+        <v>730000</v>
+      </c>
+      <c r="F114" t="s">
+        <v>365</v>
+      </c>
+      <c r="H114">
+        <v>2</v>
+      </c>
+      <c r="I114">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="115" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A115">
+        <v>114</v>
+      </c>
+      <c r="B115">
+        <v>10</v>
+      </c>
+      <c r="C115">
+        <v>10000</v>
+      </c>
+      <c r="D115" t="s">
+        <v>74</v>
+      </c>
+      <c r="E115">
+        <v>730100</v>
+      </c>
+      <c r="F115" t="s">
+        <v>112</v>
+      </c>
+      <c r="H115">
+        <v>5</v>
+      </c>
+      <c r="I115">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="116" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A116">
+        <v>115</v>
+      </c>
+      <c r="B116">
+        <v>10</v>
+      </c>
+      <c r="C116">
+        <v>10000</v>
+      </c>
+      <c r="D116" t="s">
+        <v>74</v>
+      </c>
+      <c r="E116">
+        <v>800000</v>
+      </c>
+      <c r="F116" t="s">
+        <v>368</v>
+      </c>
+      <c r="H116">
+        <v>1</v>
+      </c>
+      <c r="I116">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="117" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A117">
+        <v>116</v>
+      </c>
+      <c r="B117">
+        <v>10</v>
+      </c>
+      <c r="C117">
+        <v>10000</v>
+      </c>
+      <c r="D117" t="s">
+        <v>74</v>
+      </c>
+      <c r="E117">
+        <v>800001</v>
+      </c>
+      <c r="F117" t="s">
+        <v>366</v>
+      </c>
+      <c r="H117">
+        <v>2</v>
+      </c>
+      <c r="I117">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="118" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A118">
+        <v>117</v>
+      </c>
+      <c r="B118">
+        <v>10</v>
+      </c>
+      <c r="C118">
+        <v>10000</v>
+      </c>
+      <c r="D118" t="s">
+        <v>74</v>
+      </c>
+      <c r="E118">
+        <v>800100</v>
+      </c>
+      <c r="F118" t="s">
+        <v>113</v>
+      </c>
+      <c r="H118">
+        <v>5</v>
+      </c>
+      <c r="I118">
+        <v>426.5</v>
+      </c>
+    </row>
+    <row r="119" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A119">
+        <v>118</v>
+      </c>
+      <c r="B119">
+        <v>10</v>
+      </c>
+      <c r="C119">
+        <v>10000</v>
+      </c>
+      <c r="D119" t="s">
+        <v>74</v>
+      </c>
+      <c r="E119">
+        <v>840000</v>
+      </c>
+      <c r="F119" t="s">
+        <v>367</v>
+      </c>
+      <c r="H119">
+        <v>2</v>
+      </c>
+      <c r="I119">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="120" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A120">
+        <v>119</v>
+      </c>
+      <c r="B120">
+        <v>10</v>
+      </c>
+      <c r="C120">
+        <v>10000</v>
+      </c>
+      <c r="D120" t="s">
+        <v>74</v>
+      </c>
+      <c r="E120">
         <v>840100</v>
       </c>
-      <c r="F100" t="s">
+      <c r="F120" t="s">
         <v>114</v>
       </c>
-      <c r="H100">
-        <v>5</v>
-      </c>
-      <c r="I100">
+      <c r="H120">
+        <v>5</v>
+      </c>
+      <c r="I120">
         <v>426.5</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L99" xr:uid="{00000000-0009-0000-0000-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L99">
-      <sortCondition ref="E1:E99"/>
-    </sortState>
-  </autoFilter>
+  <autoFilter ref="A1:L120" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -4552,20 +5153,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="31" t="s">
         <v>115</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="31" t="s">
         <v>116</v>
       </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
+      <c r="B2" s="32"/>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
@@ -5089,350 +5690,350 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="31" t="s">
         <v>115</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="31" t="s">
         <v>165</v>
       </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
+      <c r="B2" s="32"/>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="27" t="s">
+      <c r="A3" s="25" t="s">
         <v>117</v>
       </c>
-      <c r="B3" s="27" t="s">
+      <c r="B3" s="25" t="s">
         <v>118</v>
       </c>
-      <c r="C3" s="27" t="s">
+      <c r="C3" s="25" t="s">
         <v>119</v>
       </c>
-      <c r="D3" s="27" t="s">
+      <c r="D3" s="25" t="s">
         <v>120</v>
       </c>
-      <c r="E3" s="28" t="s">
+      <c r="E3" s="26" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="27" t="s">
+      <c r="A4" s="25" t="s">
         <v>166</v>
       </c>
-      <c r="B4" s="29"/>
-      <c r="C4" s="29"/>
-      <c r="D4" s="29"/>
-      <c r="E4" s="30">
+      <c r="B4" s="27"/>
+      <c r="C4" s="27"/>
+      <c r="D4" s="27"/>
+      <c r="E4" s="28">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="31" t="s">
+      <c r="A5" s="29" t="s">
         <v>321</v>
       </c>
-      <c r="B5" s="32"/>
-      <c r="C5" s="32"/>
-      <c r="D5" s="32"/>
-      <c r="E5" s="32">
+      <c r="B5" s="30"/>
+      <c r="C5" s="30"/>
+      <c r="D5" s="30"/>
+      <c r="E5" s="30">
         <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="31" t="s">
+      <c r="A6" s="29" t="s">
         <v>322</v>
       </c>
-      <c r="B6" s="32"/>
-      <c r="C6" s="32"/>
-      <c r="D6" s="32"/>
-      <c r="E6" s="32">
+      <c r="B6" s="30"/>
+      <c r="C6" s="30"/>
+      <c r="D6" s="30"/>
+      <c r="E6" s="30">
         <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="31" t="s">
+      <c r="A7" s="29" t="s">
         <v>323</v>
       </c>
-      <c r="B7" s="32"/>
-      <c r="C7" s="32"/>
-      <c r="D7" s="32"/>
-      <c r="E7" s="32">
+      <c r="B7" s="30"/>
+      <c r="C7" s="30"/>
+      <c r="D7" s="30"/>
+      <c r="E7" s="30">
         <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="31" t="s">
+      <c r="A8" s="29" t="s">
         <v>324</v>
       </c>
-      <c r="B8" s="32"/>
-      <c r="C8" s="32"/>
-      <c r="D8" s="32"/>
-      <c r="E8" s="32">
+      <c r="B8" s="30"/>
+      <c r="C8" s="30"/>
+      <c r="D8" s="30"/>
+      <c r="E8" s="30">
         <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="27" t="s">
+      <c r="A9" s="25" t="s">
         <v>167</v>
       </c>
-      <c r="B9" s="29"/>
-      <c r="C9" s="29"/>
-      <c r="D9" s="29"/>
-      <c r="E9" s="30">
+      <c r="B9" s="27"/>
+      <c r="C9" s="27"/>
+      <c r="D9" s="27"/>
+      <c r="E9" s="28">
         <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="31" t="s">
+      <c r="A10" s="29" t="s">
         <v>325</v>
       </c>
-      <c r="B10" s="32"/>
-      <c r="C10" s="32"/>
-      <c r="D10" s="32"/>
-      <c r="E10" s="32">
+      <c r="B10" s="30"/>
+      <c r="C10" s="30"/>
+      <c r="D10" s="30"/>
+      <c r="E10" s="30">
         <v>2</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="31" t="s">
+      <c r="A11" s="29" t="s">
         <v>326</v>
       </c>
-      <c r="B11" s="32"/>
-      <c r="C11" s="32"/>
-      <c r="D11" s="32"/>
-      <c r="E11" s="32">
+      <c r="B11" s="30"/>
+      <c r="C11" s="30"/>
+      <c r="D11" s="30"/>
+      <c r="E11" s="30">
         <v>2</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="31" t="s">
+      <c r="A12" s="29" t="s">
         <v>327</v>
       </c>
-      <c r="B12" s="32"/>
-      <c r="C12" s="32"/>
-      <c r="D12" s="32"/>
-      <c r="E12" s="32">
+      <c r="B12" s="30"/>
+      <c r="C12" s="30"/>
+      <c r="D12" s="30"/>
+      <c r="E12" s="30">
         <v>2</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="31" t="s">
+      <c r="A13" s="29" t="s">
         <v>328</v>
       </c>
-      <c r="B13" s="32"/>
-      <c r="C13" s="32"/>
-      <c r="D13" s="32"/>
-      <c r="E13" s="32">
+      <c r="B13" s="30"/>
+      <c r="C13" s="30"/>
+      <c r="D13" s="30"/>
+      <c r="E13" s="30">
         <v>2</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="31" t="s">
+      <c r="A14" s="29" t="s">
         <v>329</v>
       </c>
-      <c r="B14" s="32"/>
-      <c r="C14" s="32"/>
-      <c r="D14" s="32"/>
-      <c r="E14" s="32">
+      <c r="B14" s="30"/>
+      <c r="C14" s="30"/>
+      <c r="D14" s="30"/>
+      <c r="E14" s="30">
         <v>2</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="31" t="s">
+      <c r="A15" s="29" t="s">
         <v>330</v>
       </c>
-      <c r="B15" s="32"/>
-      <c r="C15" s="32"/>
-      <c r="D15" s="32"/>
-      <c r="E15" s="32">
+      <c r="B15" s="30"/>
+      <c r="C15" s="30"/>
+      <c r="D15" s="30"/>
+      <c r="E15" s="30">
         <v>2</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="31" t="s">
+      <c r="A16" s="29" t="s">
         <v>331</v>
       </c>
-      <c r="B16" s="32"/>
-      <c r="C16" s="32"/>
-      <c r="D16" s="32"/>
-      <c r="E16" s="32">
+      <c r="B16" s="30"/>
+      <c r="C16" s="30"/>
+      <c r="D16" s="30"/>
+      <c r="E16" s="30">
         <v>2</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="27" t="s">
+      <c r="A17" s="25" t="s">
         <v>168</v>
       </c>
-      <c r="B17" s="29"/>
-      <c r="C17" s="29"/>
-      <c r="D17" s="29"/>
-      <c r="E17" s="30">
+      <c r="B17" s="27"/>
+      <c r="C17" s="27"/>
+      <c r="D17" s="27"/>
+      <c r="E17" s="28">
         <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="31" t="s">
+      <c r="A18" s="29" t="s">
         <v>332</v>
       </c>
-      <c r="B18" s="32"/>
-      <c r="C18" s="32"/>
-      <c r="D18" s="32"/>
-      <c r="E18" s="32">
+      <c r="B18" s="30"/>
+      <c r="C18" s="30"/>
+      <c r="D18" s="30"/>
+      <c r="E18" s="30">
         <v>2</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" s="31" t="s">
+      <c r="A19" s="29" t="s">
         <v>333</v>
       </c>
-      <c r="B19" s="32"/>
-      <c r="C19" s="32"/>
-      <c r="D19" s="32"/>
-      <c r="E19" s="32">
+      <c r="B19" s="30"/>
+      <c r="C19" s="30"/>
+      <c r="D19" s="30"/>
+      <c r="E19" s="30">
         <v>2</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="31" t="s">
+      <c r="A20" s="29" t="s">
         <v>334</v>
       </c>
-      <c r="B20" s="32"/>
-      <c r="C20" s="32"/>
-      <c r="D20" s="32"/>
-      <c r="E20" s="32">
+      <c r="B20" s="30"/>
+      <c r="C20" s="30"/>
+      <c r="D20" s="30"/>
+      <c r="E20" s="30">
         <v>2</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="31" t="s">
+      <c r="A21" s="29" t="s">
         <v>335</v>
       </c>
-      <c r="B21" s="32"/>
-      <c r="C21" s="32"/>
-      <c r="D21" s="32"/>
-      <c r="E21" s="32">
+      <c r="B21" s="30"/>
+      <c r="C21" s="30"/>
+      <c r="D21" s="30"/>
+      <c r="E21" s="30">
         <v>2</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="27" t="s">
+      <c r="A22" s="25" t="s">
         <v>169</v>
       </c>
-      <c r="B22" s="29"/>
-      <c r="C22" s="29"/>
-      <c r="D22" s="29"/>
-      <c r="E22" s="30">
+      <c r="B22" s="27"/>
+      <c r="C22" s="27"/>
+      <c r="D22" s="27"/>
+      <c r="E22" s="28">
         <v>1</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" s="31" t="s">
+      <c r="A23" s="29" t="s">
         <v>336</v>
       </c>
-      <c r="B23" s="32"/>
-      <c r="C23" s="32"/>
-      <c r="D23" s="32"/>
-      <c r="E23" s="32">
+      <c r="B23" s="30"/>
+      <c r="C23" s="30"/>
+      <c r="D23" s="30"/>
+      <c r="E23" s="30">
         <v>2</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" s="31" t="s">
+      <c r="A24" s="29" t="s">
         <v>337</v>
       </c>
-      <c r="B24" s="32"/>
-      <c r="C24" s="32"/>
-      <c r="D24" s="32"/>
-      <c r="E24" s="32">
+      <c r="B24" s="30"/>
+      <c r="C24" s="30"/>
+      <c r="D24" s="30"/>
+      <c r="E24" s="30">
         <v>2</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" s="31" t="s">
+      <c r="A25" s="29" t="s">
         <v>338</v>
       </c>
-      <c r="B25" s="32"/>
-      <c r="C25" s="32"/>
-      <c r="D25" s="32"/>
-      <c r="E25" s="32">
+      <c r="B25" s="30"/>
+      <c r="C25" s="30"/>
+      <c r="D25" s="30"/>
+      <c r="E25" s="30">
         <v>2</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" s="31" t="s">
+      <c r="A26" s="29" t="s">
         <v>339</v>
       </c>
-      <c r="B26" s="32"/>
-      <c r="C26" s="32"/>
-      <c r="D26" s="32"/>
-      <c r="E26" s="32">
+      <c r="B26" s="30"/>
+      <c r="C26" s="30"/>
+      <c r="D26" s="30"/>
+      <c r="E26" s="30">
         <v>2</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" s="27" t="s">
+      <c r="A27" s="25" t="s">
         <v>170</v>
       </c>
-      <c r="B27" s="29"/>
-      <c r="C27" s="29"/>
-      <c r="D27" s="29"/>
-      <c r="E27" s="30">
+      <c r="B27" s="27"/>
+      <c r="C27" s="27"/>
+      <c r="D27" s="27"/>
+      <c r="E27" s="28">
         <v>1</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" s="31" t="s">
+      <c r="A28" s="29" t="s">
         <v>340</v>
       </c>
-      <c r="B28" s="32"/>
-      <c r="C28" s="32"/>
-      <c r="D28" s="32"/>
-      <c r="E28" s="32">
+      <c r="B28" s="30"/>
+      <c r="C28" s="30"/>
+      <c r="D28" s="30"/>
+      <c r="E28" s="30">
         <v>2</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A29" s="31" t="s">
+      <c r="A29" s="29" t="s">
         <v>341</v>
       </c>
-      <c r="B29" s="32"/>
-      <c r="C29" s="32"/>
-      <c r="D29" s="32"/>
-      <c r="E29" s="32">
+      <c r="B29" s="30"/>
+      <c r="C29" s="30"/>
+      <c r="D29" s="30"/>
+      <c r="E29" s="30">
         <v>2</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A30" s="27" t="s">
+      <c r="A30" s="25" t="s">
         <v>342</v>
       </c>
-      <c r="B30" s="27"/>
-      <c r="C30" s="27"/>
-      <c r="D30" s="27"/>
-      <c r="E30" s="27"/>
+      <c r="B30" s="25"/>
+      <c r="C30" s="25"/>
+      <c r="D30" s="25"/>
+      <c r="E30" s="25"/>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" s="27" t="s">
+      <c r="A31" s="25" t="s">
         <v>343</v>
       </c>
-      <c r="B31" s="27"/>
-      <c r="C31" s="27"/>
-      <c r="D31" s="27"/>
-      <c r="E31" s="27"/>
+      <c r="B31" s="25"/>
+      <c r="C31" s="25"/>
+      <c r="D31" s="25"/>
+      <c r="E31" s="25"/>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" s="27" t="s">
+      <c r="A32" s="25" t="s">
         <v>344</v>
       </c>
-      <c r="B32" s="27"/>
-      <c r="C32" s="27"/>
-      <c r="D32" s="27"/>
-      <c r="E32" s="27"/>
+      <c r="B32" s="25"/>
+      <c r="C32" s="25"/>
+      <c r="D32" s="25"/>
+      <c r="E32" s="25"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -5608,39 +6209,43 @@
         <v>10</v>
       </c>
       <c r="B11" s="16">
-        <v>10100</v>
+        <v>10000</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>182</v>
+        <v>345</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="18">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="B12" s="16">
-        <v>20</v>
-      </c>
-      <c r="C12" s="16"/>
+        <v>10100</v>
+      </c>
+      <c r="C12" s="16" t="s">
+        <v>182</v>
+      </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="18">
         <v>20</v>
       </c>
       <c r="B13" s="16">
-        <v>20000</v>
-      </c>
-      <c r="C13" s="16"/>
+        <v>20</v>
+      </c>
+      <c r="C13" s="16" t="s">
+        <v>183</v>
+      </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="18">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="B14" s="16">
-        <v>30</v>
+        <v>20100</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>177</v>
+        <v>347</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -5648,16 +6253,22 @@
         <v>30</v>
       </c>
       <c r="B15" s="16">
-        <v>30000</v>
+        <v>30</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>183</v>
+        <v>346</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="18"/>
-      <c r="B16" s="16"/>
-      <c r="C16" s="16"/>
+      <c r="A16" s="18">
+        <v>30</v>
+      </c>
+      <c r="B16" s="16">
+        <v>30100</v>
+      </c>
+      <c r="C16" s="16" t="s">
+        <v>348</v>
+      </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="18"/>

</xml_diff>

<commit_message>
Feat: code-table loader, advisory context, test fixture fix (v0.1d)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/resources/Silver_Dolphins_CoA.xlsx
+++ b/resources/Silver_Dolphins_CoA.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mkc53\ClaudeProjects\Silver_Dolphins_AUDIT\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ucf-my.sharepoint.com/personal/ma755729_ucf_edu/Documents/UCF Spring 2026/AUDIT Project Files/Chart of Account/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FF0AB64-CEFB-4718-A08C-7165C51E47E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{9FF0AB64-CEFB-4718-A08C-7165C51E47E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C9B555D4-8E80-48FC-98F8-319AE0CA04A0}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="5190" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Chart of Accounts" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Feat: variable explorer traceability, VERSION sync, advisory resources (v1.0)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/resources/Silver_Dolphins_CoA.xlsx
+++ b/resources/Silver_Dolphins_CoA.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ucf-my.sharepoint.com/personal/ma755729_ucf_edu/Documents/UCF Spring 2026/AUDIT Project Files/Chart of Account/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{9FF0AB64-CEFB-4718-A08C-7165C51E47E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C9B555D4-8E80-48FC-98F8-319AE0CA04A0}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{D9323A8E-E432-4589-B17D-12A2834C5488}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FB6F092B-1D88-4078-B7A4-2C72D458668C}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="5190" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38400" yWindow="5715" windowWidth="28800" windowHeight="15885" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Chart of Accounts" sheetId="1" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="541" uniqueCount="369">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="541" uniqueCount="367">
   <si>
     <t>Account ID</t>
   </si>
@@ -574,12 +574,6 @@
   </si>
   <si>
     <t>Administrative Services</t>
-  </si>
-  <si>
-    <t>Debt Company</t>
-  </si>
-  <si>
-    <t>Operations</t>
   </si>
   <si>
     <t>Business Units</t>
@@ -1460,6 +1454,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3480,7 +3478,7 @@
         <v>400001</v>
       </c>
       <c r="F62" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="H62">
         <v>2</v>
@@ -3610,7 +3608,7 @@
         <v>420000</v>
       </c>
       <c r="F67" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="H67">
         <v>2</v>
@@ -3688,7 +3686,7 @@
         <v>450000</v>
       </c>
       <c r="F70" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="H70">
         <v>2</v>
@@ -3795,7 +3793,7 @@
         <v>500001</v>
       </c>
       <c r="F74" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="H74">
         <v>2</v>
@@ -3899,7 +3897,7 @@
         <v>510000</v>
       </c>
       <c r="F78" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="H78">
         <v>2</v>
@@ -4029,7 +4027,7 @@
         <v>530000</v>
       </c>
       <c r="F83" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="H83">
         <v>2</v>
@@ -4185,7 +4183,7 @@
         <v>540000</v>
       </c>
       <c r="F89" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="H89">
         <v>2</v>
@@ -4263,7 +4261,7 @@
         <v>550000</v>
       </c>
       <c r="F92" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="H92">
         <v>2</v>
@@ -4419,7 +4417,7 @@
         <v>570000</v>
       </c>
       <c r="F98" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="H98">
         <v>2</v>
@@ -4471,7 +4469,7 @@
         <v>580000</v>
       </c>
       <c r="F100" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="H100">
         <v>2</v>
@@ -4526,7 +4524,7 @@
         <v>600001</v>
       </c>
       <c r="F102" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="H102">
         <v>2</v>
@@ -4578,7 +4576,7 @@
         <v>610000</v>
       </c>
       <c r="F104" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="H104">
         <v>2</v>
@@ -4630,7 +4628,7 @@
         <v>620000</v>
       </c>
       <c r="F106" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="H106">
         <v>2</v>
@@ -4682,7 +4680,7 @@
         <v>630000</v>
       </c>
       <c r="F108" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="H108">
         <v>2</v>
@@ -4708,7 +4706,7 @@
         <v>700001</v>
       </c>
       <c r="F109" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="H109">
         <v>2</v>
@@ -4815,7 +4813,7 @@
         <v>720000</v>
       </c>
       <c r="F113" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="H113">
         <v>2</v>
@@ -4841,7 +4839,7 @@
         <v>730000</v>
       </c>
       <c r="F114" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="H114">
         <v>2</v>
@@ -4893,7 +4891,7 @@
         <v>800000</v>
       </c>
       <c r="F116" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="H116">
         <v>1</v>
@@ -4919,7 +4917,7 @@
         <v>800001</v>
       </c>
       <c r="F117" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="H117">
         <v>2</v>
@@ -4971,7 +4969,7 @@
         <v>840000</v>
       </c>
       <c r="F119" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="H119">
         <v>2</v>
@@ -5037,33 +5035,33 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="21" t="s">
+        <v>184</v>
+      </c>
+      <c r="B9" s="22" t="s">
+        <v>185</v>
+      </c>
+      <c r="C9" s="22" t="s">
         <v>186</v>
-      </c>
-      <c r="B9" s="22" t="s">
-        <v>187</v>
-      </c>
-      <c r="C9" s="22" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="18"/>
       <c r="B10" s="16" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="18" t="s">
+        <v>311</v>
+      </c>
+      <c r="B11" s="16" t="s">
+        <v>312</v>
+      </c>
+      <c r="C11" s="16" t="s">
         <v>313</v>
-      </c>
-      <c r="B11" s="16" t="s">
-        <v>314</v>
-      </c>
-      <c r="C11" s="16" t="s">
-        <v>315</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -5071,21 +5069,21 @@
         <v>21</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="18" t="s">
+        <v>316</v>
+      </c>
+      <c r="B13" s="16" t="s">
+        <v>317</v>
+      </c>
+      <c r="C13" s="16" t="s">
         <v>318</v>
-      </c>
-      <c r="B13" s="16" t="s">
-        <v>319</v>
-      </c>
-      <c r="C13" s="16" t="s">
-        <v>320</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -5735,7 +5733,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="29" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="B5" s="30"/>
       <c r="C5" s="30"/>
@@ -5746,7 +5744,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="29" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="B6" s="30"/>
       <c r="C6" s="30"/>
@@ -5757,7 +5755,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="29" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="B7" s="30"/>
       <c r="C7" s="30"/>
@@ -5768,7 +5766,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="29" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="B8" s="30"/>
       <c r="C8" s="30"/>
@@ -5790,7 +5788,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="29" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="B10" s="30"/>
       <c r="C10" s="30"/>
@@ -5801,7 +5799,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="29" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="B11" s="30"/>
       <c r="C11" s="30"/>
@@ -5812,7 +5810,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="29" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="B12" s="30"/>
       <c r="C12" s="30"/>
@@ -5823,7 +5821,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="29" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="B13" s="30"/>
       <c r="C13" s="30"/>
@@ -5834,7 +5832,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="29" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="B14" s="30"/>
       <c r="C14" s="30"/>
@@ -5845,7 +5843,7 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="29" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="B15" s="30"/>
       <c r="C15" s="30"/>
@@ -5856,7 +5854,7 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="29" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="B16" s="30"/>
       <c r="C16" s="30"/>
@@ -5878,7 +5876,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="29" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="B18" s="30"/>
       <c r="C18" s="30"/>
@@ -5889,7 +5887,7 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="29" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="B19" s="30"/>
       <c r="C19" s="30"/>
@@ -5900,7 +5898,7 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="29" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="B20" s="30"/>
       <c r="C20" s="30"/>
@@ -5911,7 +5909,7 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="29" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="B21" s="30"/>
       <c r="C21" s="30"/>
@@ -5933,7 +5931,7 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="29" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="B23" s="30"/>
       <c r="C23" s="30"/>
@@ -5944,7 +5942,7 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="29" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="B24" s="30"/>
       <c r="C24" s="30"/>
@@ -5955,7 +5953,7 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="29" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="B25" s="30"/>
       <c r="C25" s="30"/>
@@ -5966,7 +5964,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="29" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="B26" s="30"/>
       <c r="C26" s="30"/>
@@ -5988,7 +5986,7 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="29" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="B28" s="30"/>
       <c r="C28" s="30"/>
@@ -5999,7 +5997,7 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="29" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="B29" s="30"/>
       <c r="C29" s="30"/>
@@ -6010,7 +6008,7 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="25" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="B30" s="25"/>
       <c r="C30" s="25"/>
@@ -6019,7 +6017,7 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="25" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="B31" s="25"/>
       <c r="C31" s="25"/>
@@ -6028,7 +6026,7 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="25" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="B32" s="25"/>
       <c r="C32" s="25"/>
@@ -6091,7 +6089,7 @@
         <v>20</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="C11" s="16"/>
     </row>
@@ -6100,7 +6098,7 @@
         <v>30</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>177</v>
+        <v>344</v>
       </c>
       <c r="C12" s="16"/>
     </row>
@@ -6174,7 +6172,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -6184,13 +6182,13 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="23" t="s">
+        <v>177</v>
+      </c>
+      <c r="B9" s="23" t="s">
+        <v>178</v>
+      </c>
+      <c r="C9" s="24" t="s">
         <v>179</v>
-      </c>
-      <c r="B9" s="23" t="s">
-        <v>180</v>
-      </c>
-      <c r="C9" s="24" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -6212,7 +6210,7 @@
         <v>10000</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -6223,7 +6221,7 @@
         <v>10100</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -6234,7 +6232,7 @@
         <v>20</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -6245,7 +6243,7 @@
         <v>20100</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -6256,7 +6254,7 @@
         <v>30</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -6267,7 +6265,7 @@
         <v>30100</v>
       </c>
       <c r="C16" s="16" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -6320,7 +6318,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -6328,27 +6326,27 @@
         <v>172</v>
       </c>
       <c r="B3" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="21" t="s">
+        <v>184</v>
+      </c>
+      <c r="B9" s="22" t="s">
+        <v>185</v>
+      </c>
+      <c r="C9" s="22" t="s">
         <v>186</v>
-      </c>
-      <c r="B9" s="22" t="s">
-        <v>187</v>
-      </c>
-      <c r="C9" s="22" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="18"/>
       <c r="B10" s="16" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -6356,32 +6354,32 @@
         <v>14</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="18" t="s">
+        <v>191</v>
+      </c>
+      <c r="B12" s="16" t="s">
+        <v>192</v>
+      </c>
+      <c r="C12" s="16" t="s">
         <v>193</v>
-      </c>
-      <c r="B12" s="16" t="s">
-        <v>194</v>
-      </c>
-      <c r="C12" s="16" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="18" t="s">
+        <v>194</v>
+      </c>
+      <c r="B13" s="16" t="s">
+        <v>195</v>
+      </c>
+      <c r="C13" s="16" t="s">
         <v>196</v>
-      </c>
-      <c r="B13" s="16" t="s">
-        <v>197</v>
-      </c>
-      <c r="C13" s="16" t="s">
-        <v>198</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -6449,7 +6447,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -6459,13 +6457,13 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="19" t="s">
+        <v>184</v>
+      </c>
+      <c r="B9" s="19" t="s">
+        <v>185</v>
+      </c>
+      <c r="C9" s="20" t="s">
         <v>186</v>
-      </c>
-      <c r="B9" s="19" t="s">
-        <v>187</v>
-      </c>
-      <c r="C9" s="20" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -6473,7 +6471,7 @@
         <v>101</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="C10" s="16"/>
     </row>
@@ -6482,7 +6480,7 @@
         <v>101.1</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="C11" s="16"/>
     </row>
@@ -6491,7 +6489,7 @@
         <v>107</v>
       </c>
       <c r="B12" s="18" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="C12" s="16"/>
     </row>
@@ -6500,7 +6498,7 @@
         <v>108</v>
       </c>
       <c r="B13" s="18" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="C13" s="16"/>
     </row>
@@ -6509,7 +6507,7 @@
         <v>111</v>
       </c>
       <c r="B14" s="18" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="C14" s="16"/>
     </row>
@@ -6518,7 +6516,7 @@
         <v>114</v>
       </c>
       <c r="B15" s="18" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="C15" s="16"/>
     </row>
@@ -6527,7 +6525,7 @@
         <v>124</v>
       </c>
       <c r="B16" s="18" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="C16" s="16"/>
     </row>
@@ -6536,7 +6534,7 @@
         <v>128</v>
       </c>
       <c r="B17" s="18" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="C17" s="16"/>
     </row>
@@ -6545,7 +6543,7 @@
         <v>131</v>
       </c>
       <c r="B18" s="18" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="C18" s="16"/>
     </row>
@@ -6554,7 +6552,7 @@
         <v>142</v>
       </c>
       <c r="B19" s="18" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="C19" s="16"/>
     </row>
@@ -6563,7 +6561,7 @@
         <v>151</v>
       </c>
       <c r="B20" s="18" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="C20" s="16"/>
     </row>
@@ -6572,7 +6570,7 @@
         <v>154</v>
       </c>
       <c r="B21" s="18" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="C21" s="16"/>
     </row>
@@ -6581,7 +6579,7 @@
         <v>165</v>
       </c>
       <c r="B22" s="18" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="C22" s="16"/>
     </row>
@@ -6590,7 +6588,7 @@
         <v>173</v>
       </c>
       <c r="B23" s="18" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="C23" s="16"/>
     </row>
@@ -6599,7 +6597,7 @@
         <v>201</v>
       </c>
       <c r="B24" s="18" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C24" s="16"/>
     </row>
@@ -6608,7 +6606,7 @@
         <v>211</v>
       </c>
       <c r="B25" s="18" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="C25" s="16"/>
     </row>
@@ -6617,7 +6615,7 @@
         <v>216</v>
       </c>
       <c r="B26" s="18" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="C26" s="16"/>
     </row>
@@ -6626,7 +6624,7 @@
         <v>221</v>
       </c>
       <c r="B27" s="18" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="C27" s="16"/>
     </row>
@@ -6635,7 +6633,7 @@
         <v>228.3</v>
       </c>
       <c r="B28" s="18" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="C28" s="16"/>
     </row>
@@ -6644,7 +6642,7 @@
         <v>228.4</v>
       </c>
       <c r="B29" s="18" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="C29" s="16"/>
     </row>
@@ -6653,7 +6651,7 @@
         <v>232</v>
       </c>
       <c r="B30" s="18" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="C30" s="16"/>
     </row>
@@ -6662,7 +6660,7 @@
         <v>235</v>
       </c>
       <c r="B31" s="18" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="C31" s="16"/>
     </row>
@@ -6671,7 +6669,7 @@
         <v>236</v>
       </c>
       <c r="B32" s="18" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="C32" s="16"/>
     </row>
@@ -6680,7 +6678,7 @@
         <v>237</v>
       </c>
       <c r="B33" s="18" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="C33" s="16"/>
     </row>
@@ -6689,7 +6687,7 @@
         <v>242</v>
       </c>
       <c r="B34" s="18" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="C34" s="16"/>
     </row>
@@ -6698,7 +6696,7 @@
         <v>302</v>
       </c>
       <c r="B35" s="18" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="C35" s="16"/>
     </row>
@@ -6707,7 +6705,7 @@
         <v>303</v>
       </c>
       <c r="B36" s="18" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="C36" s="16"/>
     </row>
@@ -6716,7 +6714,7 @@
         <v>310</v>
       </c>
       <c r="B37" s="18" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="C37" s="16"/>
     </row>
@@ -6725,7 +6723,7 @@
         <v>311</v>
       </c>
       <c r="B38" s="18" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C38" s="16"/>
     </row>
@@ -6734,7 +6732,7 @@
         <v>314</v>
       </c>
       <c r="B39" s="18" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C39" s="16"/>
     </row>
@@ -6743,7 +6741,7 @@
         <v>355</v>
       </c>
       <c r="B40" s="18" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="C40" s="16"/>
     </row>
@@ -6752,7 +6750,7 @@
         <v>370</v>
       </c>
       <c r="B41" s="18" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="C41" s="16"/>
     </row>
@@ -6761,7 +6759,7 @@
         <v>400</v>
       </c>
       <c r="B42" s="18" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="C42" s="16"/>
     </row>
@@ -6770,7 +6768,7 @@
         <v>403</v>
       </c>
       <c r="B43" s="18" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="C43" s="16"/>
     </row>
@@ -6779,7 +6777,7 @@
         <v>404</v>
       </c>
       <c r="B44" s="18" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="C44" s="16"/>
     </row>
@@ -6788,7 +6786,7 @@
         <v>407.3</v>
       </c>
       <c r="B45" s="18" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="C45" s="16"/>
     </row>
@@ -6797,7 +6795,7 @@
         <v>408.1</v>
       </c>
       <c r="B46" s="18" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="C46" s="16"/>
     </row>
@@ -6806,7 +6804,7 @@
         <v>418</v>
       </c>
       <c r="B47" s="18" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="C47" s="16"/>
     </row>
@@ -6815,7 +6813,7 @@
         <v>419</v>
       </c>
       <c r="B48" s="18" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="C48" s="16"/>
     </row>
@@ -6824,7 +6822,7 @@
         <v>421</v>
       </c>
       <c r="B49" s="18" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="C49" s="16"/>
     </row>
@@ -6833,7 +6831,7 @@
         <v>426.5</v>
       </c>
       <c r="B50" s="18" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="C50" s="16"/>
     </row>
@@ -6842,7 +6840,7 @@
         <v>427</v>
       </c>
       <c r="B51" s="18" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C51" s="16"/>
     </row>
@@ -6851,7 +6849,7 @@
         <v>428</v>
       </c>
       <c r="B52" s="18" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="C52" s="16"/>
     </row>
@@ -6860,7 +6858,7 @@
         <v>438</v>
       </c>
       <c r="B53" s="18" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="C53" s="16"/>
     </row>
@@ -6869,7 +6867,7 @@
         <v>440</v>
       </c>
       <c r="B54" s="18" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="C54" s="16"/>
     </row>
@@ -6878,7 +6876,7 @@
         <v>442</v>
       </c>
       <c r="B55" s="18" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="C55" s="16"/>
     </row>
@@ -6887,7 +6885,7 @@
         <v>447</v>
       </c>
       <c r="B56" s="18" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="C56" s="16"/>
     </row>
@@ -6896,7 +6894,7 @@
         <v>450</v>
       </c>
       <c r="B57" s="18" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="C57" s="16"/>
     </row>
@@ -6905,7 +6903,7 @@
         <v>456</v>
       </c>
       <c r="B58" s="18" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="C58" s="16"/>
     </row>
@@ -6914,7 +6912,7 @@
         <v>500</v>
       </c>
       <c r="B59" s="18" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="C59" s="16"/>
     </row>
@@ -6923,7 +6921,7 @@
         <v>501</v>
       </c>
       <c r="B60" s="18" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="C60" s="16"/>
     </row>
@@ -6932,7 +6930,7 @@
         <v>506</v>
       </c>
       <c r="B61" s="18" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="C61" s="16"/>
     </row>
@@ -6941,7 +6939,7 @@
         <v>555</v>
       </c>
       <c r="B62" s="18" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="C62" s="16"/>
     </row>
@@ -6950,7 +6948,7 @@
         <v>571</v>
       </c>
       <c r="B63" s="18" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="C63" s="16"/>
     </row>
@@ -6959,7 +6957,7 @@
         <v>593</v>
       </c>
       <c r="B64" s="18" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="C64" s="16"/>
     </row>
@@ -6968,7 +6966,7 @@
         <v>920</v>
       </c>
       <c r="B65" s="18" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="C65" s="16"/>
     </row>
@@ -6977,7 +6975,7 @@
         <v>921</v>
       </c>
       <c r="B66" s="18" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="C66" s="16"/>
     </row>
@@ -6986,7 +6984,7 @@
         <v>923</v>
       </c>
       <c r="B67" s="18" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="C67" s="16"/>
     </row>
@@ -6995,7 +6993,7 @@
         <v>926</v>
       </c>
       <c r="B68" s="18" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="C68" s="16"/>
     </row>
@@ -7004,7 +7002,7 @@
         <v>998</v>
       </c>
       <c r="B69" s="18" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C69" s="16"/>
     </row>
@@ -7013,7 +7011,7 @@
         <v>999</v>
       </c>
       <c r="B70" s="18" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="C70" s="16"/>
     </row>
@@ -7080,7 +7078,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -7090,110 +7088,110 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="19" t="s">
+        <v>184</v>
+      </c>
+      <c r="B9" s="19" t="s">
+        <v>185</v>
+      </c>
+      <c r="C9" s="20" t="s">
         <v>186</v>
-      </c>
-      <c r="B9" s="19" t="s">
-        <v>187</v>
-      </c>
-      <c r="C9" s="20" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="18"/>
       <c r="B10" s="18" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="18" t="s">
+        <v>261</v>
+      </c>
+      <c r="B11" s="18" t="s">
+        <v>262</v>
+      </c>
+      <c r="C11" s="16" t="s">
         <v>263</v>
-      </c>
-      <c r="B11" s="18" t="s">
-        <v>264</v>
-      </c>
-      <c r="C11" s="16" t="s">
-        <v>265</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="18" t="s">
+        <v>264</v>
+      </c>
+      <c r="B12" s="18" t="s">
+        <v>265</v>
+      </c>
+      <c r="C12" s="16" t="s">
         <v>266</v>
-      </c>
-      <c r="B12" s="18" t="s">
-        <v>267</v>
-      </c>
-      <c r="C12" s="16" t="s">
-        <v>268</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="18" t="s">
+        <v>267</v>
+      </c>
+      <c r="B13" s="18" t="s">
+        <v>268</v>
+      </c>
+      <c r="C13" s="16" t="s">
         <v>269</v>
-      </c>
-      <c r="B13" s="18" t="s">
-        <v>270</v>
-      </c>
-      <c r="C13" s="16" t="s">
-        <v>271</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="18" t="s">
+        <v>270</v>
+      </c>
+      <c r="B14" s="18" t="s">
+        <v>271</v>
+      </c>
+      <c r="C14" s="16" t="s">
         <v>272</v>
-      </c>
-      <c r="B14" s="18" t="s">
-        <v>273</v>
-      </c>
-      <c r="C14" s="16" t="s">
-        <v>274</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="18" t="s">
+        <v>273</v>
+      </c>
+      <c r="B15" s="18" t="s">
+        <v>274</v>
+      </c>
+      <c r="C15" s="16" t="s">
         <v>275</v>
-      </c>
-      <c r="B15" s="18" t="s">
-        <v>276</v>
-      </c>
-      <c r="C15" s="16" t="s">
-        <v>277</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="18" t="s">
+        <v>276</v>
+      </c>
+      <c r="B16" s="18" t="s">
+        <v>277</v>
+      </c>
+      <c r="C16" s="16" t="s">
         <v>278</v>
-      </c>
-      <c r="B16" s="18" t="s">
-        <v>279</v>
-      </c>
-      <c r="C16" s="16" t="s">
-        <v>280</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="18" t="s">
+        <v>279</v>
+      </c>
+      <c r="B17" s="18" t="s">
+        <v>280</v>
+      </c>
+      <c r="C17" s="16" t="s">
         <v>281</v>
-      </c>
-      <c r="B17" s="18" t="s">
-        <v>282</v>
-      </c>
-      <c r="C17" s="16" t="s">
-        <v>283</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="17" t="s">
+        <v>282</v>
+      </c>
+      <c r="B18" s="17" t="s">
+        <v>283</v>
+      </c>
+      <c r="C18" s="15" t="s">
         <v>284</v>
-      </c>
-      <c r="B18" s="17" t="s">
-        <v>285</v>
-      </c>
-      <c r="C18" s="15" t="s">
-        <v>286</v>
       </c>
     </row>
   </sheetData>
@@ -7216,7 +7214,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -7226,22 +7224,22 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="21" t="s">
+        <v>184</v>
+      </c>
+      <c r="B9" s="22" t="s">
+        <v>185</v>
+      </c>
+      <c r="C9" s="22" t="s">
         <v>186</v>
-      </c>
-      <c r="B9" s="22" t="s">
-        <v>187</v>
-      </c>
-      <c r="C9" s="22" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="18"/>
       <c r="B10" s="16" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -7249,10 +7247,10 @@
         <v>0</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -7260,10 +7258,10 @@
         <v>36</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -7271,10 +7269,10 @@
         <v>48</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -7282,10 +7280,10 @@
         <v>60</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -7293,10 +7291,10 @@
         <v>84</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -7304,10 +7302,10 @@
         <v>120</v>
       </c>
       <c r="B16" s="16" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="C16" s="16" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -7315,10 +7313,10 @@
         <v>300</v>
       </c>
       <c r="B17" s="16" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="C17" s="16" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -7326,10 +7324,10 @@
         <v>360</v>
       </c>
       <c r="B18" s="16" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="C18" s="16" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
@@ -7337,10 +7335,10 @@
         <v>420</v>
       </c>
       <c r="B19" s="16" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="C19" s="16" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
@@ -7348,10 +7346,10 @@
         <v>480</v>
       </c>
       <c r="B20" s="16" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="C20" s="16" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -7359,10 +7357,10 @@
         <v>540</v>
       </c>
       <c r="B21" s="16" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="C21" s="16" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -7370,10 +7368,10 @@
         <v>600</v>
       </c>
       <c r="B22" s="15" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="C22" s="15" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
     </row>
   </sheetData>

</xml_diff>